<commit_message>
Add summary results and requirements for Dyno Investigation; update isolation diagram and efficiency comparison files
- Created SummaryResults.csv to log dyno test results.
- Added requirements.txt for necessary Python packages (numpy, pandas, matplotlib, scipy).
- Updated Isolation Diagram.drawio with new version and layout adjustments.
- Updated Efficiency Comparison.xlsx with new data.
- Added Isolation Diagram.drawio.png as a visual representation of the isolation diagram.
</commit_message>
<xml_diff>
--- a/Write Ups/PowerElectronics/Efficiency Comparison.xlsx
+++ b/Write Ups/PowerElectronics/Efficiency Comparison.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Masters\Project\Write Ups\PowerElectronics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conor\Documents\College\Masters\Thesis\GeecPE2526\Write Ups\PowerElectronics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6FACD90-23B8-40E5-A7E2-240C014C444D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3692F02-DE93-495E-A1DF-629B4DAA43BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5160" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="amCharts" sheetId="1" r:id="rId1"/>
@@ -92,10 +92,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -223,7 +221,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="4"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
@@ -676,7 +674,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="4"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
@@ -1129,7 +1127,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="4"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent3"/>
@@ -1576,13 +1574,14 @@
               <a:solidFill>
                 <a:schemeClr val="accent4"/>
               </a:solidFill>
+              <a:prstDash val="dash"/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="4"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent4"/>
@@ -2029,13 +2028,14 @@
               <a:solidFill>
                 <a:schemeClr val="accent5"/>
               </a:solidFill>
+              <a:prstDash val="dash"/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="4"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent5"/>
@@ -2482,21 +2482,20 @@
               <a:solidFill>
                 <a:schemeClr val="accent6"/>
               </a:solidFill>
+              <a:prstDash val="dash"/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="4"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent6"/>
               </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent6"/>
-                </a:solidFill>
+              <a:ln w="3175">
+                <a:noFill/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
@@ -2932,7 +2931,7 @@
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
-          <c:max val="0.30000000000000004"/>
+          <c:max val="2"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -3083,6 +3082,20 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="5000"/>
+                  <a:lumOff val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:minorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -3828,10 +3841,10 @@
       <xdr:rowOff>104774</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>85724</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>19049</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4189,7 +4202,7 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>5</v>
       </c>
       <c r="C1" t="s">
@@ -4198,13 +4211,13 @@
       <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -4221,13 +4234,13 @@
       <c r="D2">
         <v>82.022999999999996</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2">
         <v>84.819000000000003</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2">
         <v>82.424999999999997</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>79.972999999999999</v>
       </c>
     </row>
@@ -4244,13 +4257,13 @@
       <c r="D3">
         <v>86.317999999999998</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3">
         <v>88.772000000000006</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3">
         <v>86.557000000000002</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>84.239000000000004</v>
       </c>
     </row>
@@ -4267,13 +4280,13 @@
       <c r="D4">
         <v>88.638999999999996</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <v>90.89</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4">
         <v>88.783000000000001</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>86.548000000000002</v>
       </c>
     </row>
@@ -4290,13 +4303,13 @@
       <c r="D5">
         <v>90.091999999999999</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5">
         <v>92.21</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5">
         <v>90.174000000000007</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5">
         <v>87.995000000000005</v>
       </c>
     </row>
@@ -4313,13 +4326,13 @@
       <c r="D6">
         <v>91.087999999999994</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6">
         <v>93.111999999999995</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6">
         <v>91.125</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6">
         <v>88.986000000000004</v>
       </c>
     </row>
@@ -4336,13 +4349,13 @@
       <c r="D7">
         <v>91.813000000000002</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7">
         <v>93.766000000000005</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7">
         <v>91.817999999999998</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7">
         <v>89.709000000000003</v>
       </c>
     </row>
@@ -4359,13 +4372,13 @@
       <c r="D8">
         <v>92.364000000000004</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8">
         <v>94.263000000000005</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8">
         <v>92.343999999999994</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8">
         <v>90.257999999999996</v>
       </c>
     </row>
@@ -4382,13 +4395,13 @@
       <c r="D9">
         <v>92.796999999999997</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9">
         <v>94.653999999999996</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9">
         <v>92.757000000000005</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9">
         <v>90.69</v>
       </c>
     </row>
@@ -4405,13 +4418,13 @@
       <c r="D10">
         <v>93.147000000000006</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10">
         <v>94.968000000000004</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10">
         <v>93.09</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10">
         <v>91.037999999999997</v>
       </c>
     </row>
@@ -4428,13 +4441,13 @@
       <c r="D11">
         <v>93.435000000000002</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11">
         <v>95.227000000000004</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11">
         <v>93.364999999999995</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11">
         <v>91.325999999999993</v>
       </c>
     </row>
@@ -4451,13 +4464,13 @@
       <c r="D12">
         <v>93.676000000000002</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12">
         <v>95.444000000000003</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12">
         <v>93.594999999999999</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12">
         <v>91.566000000000003</v>
       </c>
     </row>
@@ -4474,13 +4487,13 @@
       <c r="D13">
         <v>93.881</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13">
         <v>95.629000000000005</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13">
         <v>93.79</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13">
         <v>91.771000000000001</v>
       </c>
     </row>
@@ -4497,13 +4510,13 @@
       <c r="D14">
         <v>94.058000000000007</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14">
         <v>95.787000000000006</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14">
         <v>93.959000000000003</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14">
         <v>91.947000000000003</v>
       </c>
     </row>
@@ -4520,13 +4533,13 @@
       <c r="D15">
         <v>94.212000000000003</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15">
         <v>95.924999999999997</v>
       </c>
-      <c r="F15" s="1">
+      <c r="F15">
         <v>94.105000000000004</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15">
         <v>92.1</v>
       </c>
     </row>
@@ -4543,13 +4556,13 @@
       <c r="D16">
         <v>94.346000000000004</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16">
         <v>96.046000000000006</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16">
         <v>94.233000000000004</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16">
         <v>92.234999999999999</v>
       </c>
     </row>
@@ -4566,13 +4579,13 @@
       <c r="D17">
         <v>94.465999999999994</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17">
         <v>96.153000000000006</v>
       </c>
-      <c r="F17" s="1">
+      <c r="F17">
         <v>94.346999999999994</v>
       </c>
-      <c r="G17" s="1">
+      <c r="G17">
         <v>92.353999999999999</v>
       </c>
     </row>
@@ -4589,13 +4602,13 @@
       <c r="D18">
         <v>94.572000000000003</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18">
         <v>96.248000000000005</v>
       </c>
-      <c r="F18" s="1">
+      <c r="F18">
         <v>94.447999999999993</v>
       </c>
-      <c r="G18" s="1">
+      <c r="G18">
         <v>92.46</v>
       </c>
     </row>
@@ -4612,13 +4625,13 @@
       <c r="D19">
         <v>94.667000000000002</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19">
         <v>96.332999999999998</v>
       </c>
-      <c r="F19" s="1">
+      <c r="F19">
         <v>94.539000000000001</v>
       </c>
-      <c r="G19" s="1">
+      <c r="G19">
         <v>92.555000000000007</v>
       </c>
     </row>
@@ -4635,13 +4648,13 @@
       <c r="D20">
         <v>94.753</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20">
         <v>96.41</v>
       </c>
-      <c r="F20" s="1">
+      <c r="F20">
         <v>94.620999999999995</v>
       </c>
-      <c r="G20" s="1">
+      <c r="G20">
         <v>92.64</v>
       </c>
     </row>
@@ -4658,13 +4671,13 @@
       <c r="D21">
         <v>95.301000000000002</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21">
         <v>96.900999999999996</v>
       </c>
-      <c r="F21" s="1">
+      <c r="F21">
         <v>95.141999999999996</v>
       </c>
-      <c r="G21" s="1">
+      <c r="G21">
         <v>93.186999999999998</v>
       </c>
     </row>
@@ -4681,13 +4694,13 @@
       <c r="D22">
         <v>95.576999999999998</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22">
         <v>97.147999999999996</v>
       </c>
-      <c r="F22" s="1">
+      <c r="F22">
         <v>95.403999999999996</v>
       </c>
-      <c r="G22" s="1">
+      <c r="G22">
         <v>93.462000000000003</v>
       </c>
     </row>
@@ -4704,13 +4717,13 @@
       <c r="D23">
         <v>95.744</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23">
         <v>97.296999999999997</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F23">
         <v>95.563000000000002</v>
       </c>
-      <c r="G23" s="1">
+      <c r="G23">
         <v>93.628</v>
       </c>
     </row>
@@ -4727,13 +4740,13 @@
       <c r="D24">
         <v>95.855000000000004</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24">
         <v>97.396000000000001</v>
       </c>
-      <c r="F24" s="1">
+      <c r="F24">
         <v>95.668000000000006</v>
       </c>
-      <c r="G24" s="1">
+      <c r="G24">
         <v>93.739000000000004</v>
       </c>
     </row>
@@ -4750,13 +4763,13 @@
       <c r="D25">
         <v>95.933999999999997</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25">
         <v>97.466999999999999</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25">
         <v>95.744</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25">
         <v>93.817999999999998</v>
       </c>
     </row>
@@ -4773,13 +4786,13 @@
       <c r="D26">
         <v>95.994</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26">
         <v>97.521000000000001</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26">
         <v>95.801000000000002</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G26">
         <v>93.876999999999995</v>
       </c>
     </row>
@@ -4796,13 +4809,13 @@
       <c r="D27">
         <v>96.040999999999997</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27">
         <v>97.563000000000002</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F27">
         <v>95.844999999999999</v>
       </c>
-      <c r="G27" s="1">
+      <c r="G27">
         <v>93.924000000000007</v>
       </c>
     </row>
@@ -4819,13 +4832,13 @@
       <c r="D28">
         <v>96.078000000000003</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28">
         <v>97.596000000000004</v>
       </c>
-      <c r="F28" s="1">
+      <c r="F28">
         <v>95.88</v>
       </c>
-      <c r="G28" s="1">
+      <c r="G28">
         <v>93.96</v>
       </c>
     </row>
@@ -4842,13 +4855,13 @@
       <c r="D29">
         <v>96.108000000000004</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29">
         <v>97.623000000000005</v>
       </c>
-      <c r="F29" s="1">
+      <c r="F29">
         <v>95.909000000000006</v>
       </c>
-      <c r="G29" s="1">
+      <c r="G29">
         <v>93.99</v>
       </c>
     </row>
@@ -4865,13 +4878,13 @@
       <c r="D30">
         <v>96.134</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30">
         <v>97.646000000000001</v>
       </c>
-      <c r="F30" s="1">
+      <c r="F30">
         <v>95.933000000000007</v>
       </c>
-      <c r="G30" s="1">
+      <c r="G30">
         <v>94.016000000000005</v>
       </c>
     </row>
@@ -4888,13 +4901,13 @@
       <c r="D31">
         <v>96.155000000000001</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31">
         <v>97.665000000000006</v>
       </c>
-      <c r="F31" s="1">
+      <c r="F31">
         <v>95.953000000000003</v>
       </c>
-      <c r="G31" s="1">
+      <c r="G31">
         <v>94.037000000000006</v>
       </c>
     </row>
@@ -4911,13 +4924,13 @@
       <c r="D32">
         <v>96.174000000000007</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32">
         <v>97.682000000000002</v>
       </c>
-      <c r="F32" s="1">
+      <c r="F32">
         <v>95.971000000000004</v>
       </c>
-      <c r="G32" s="1">
+      <c r="G32">
         <v>94.055000000000007</v>
       </c>
     </row>
@@ -4934,13 +4947,13 @@
       <c r="D33">
         <v>96.19</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33">
         <v>97.695999999999998</v>
       </c>
-      <c r="F33" s="1">
+      <c r="F33">
         <v>95.986000000000004</v>
       </c>
-      <c r="G33" s="1">
+      <c r="G33">
         <v>94.07</v>
       </c>
     </row>
@@ -4957,13 +4970,13 @@
       <c r="D34">
         <v>96.203000000000003</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34">
         <v>97.709000000000003</v>
       </c>
-      <c r="F34" s="1">
+      <c r="F34">
         <v>95.998999999999995</v>
       </c>
-      <c r="G34" s="1">
+      <c r="G34">
         <v>94.084000000000003</v>
       </c>
     </row>
@@ -4980,13 +4993,13 @@
       <c r="D35">
         <v>96.215999999999994</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35">
         <v>97.72</v>
       </c>
-      <c r="F35" s="1">
+      <c r="F35">
         <v>96.01</v>
       </c>
-      <c r="G35" s="1">
+      <c r="G35">
         <v>94.096000000000004</v>
       </c>
     </row>
@@ -5003,13 +5016,13 @@
       <c r="D36">
         <v>96.227000000000004</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36">
         <v>97.728999999999999</v>
       </c>
-      <c r="F36" s="1">
+      <c r="F36">
         <v>96.021000000000001</v>
       </c>
-      <c r="G36" s="1">
+      <c r="G36">
         <v>94.106999999999999</v>
       </c>
     </row>
@@ -5026,13 +5039,13 @@
       <c r="D37">
         <v>96.236000000000004</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37">
         <v>97.738</v>
       </c>
-      <c r="F37" s="1">
+      <c r="F37">
         <v>96.03</v>
       </c>
-      <c r="G37" s="1">
+      <c r="G37">
         <v>94.116</v>
       </c>
     </row>
@@ -5049,13 +5062,13 @@
       <c r="D38">
         <v>96.245000000000005</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38">
         <v>97.745999999999995</v>
       </c>
-      <c r="F38" s="1">
+      <c r="F38">
         <v>96.037999999999997</v>
       </c>
-      <c r="G38" s="1">
+      <c r="G38">
         <v>94.123999999999995</v>
       </c>
     </row>
@@ -5072,13 +5085,13 @@
       <c r="D39">
         <v>96.3</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39">
         <v>97.796000000000006</v>
       </c>
-      <c r="F39" s="1">
+      <c r="F39">
         <v>96.09</v>
       </c>
-      <c r="G39" s="1">
+      <c r="G39">
         <v>94.177000000000007</v>
       </c>
     </row>
@@ -5095,13 +5108,13 @@
       <c r="D40">
         <v>96.328000000000003</v>
       </c>
-      <c r="E40" s="1">
+      <c r="E40">
         <v>97.820999999999998</v>
       </c>
-      <c r="F40" s="1">
+      <c r="F40">
         <v>96.114000000000004</v>
       </c>
-      <c r="G40" s="1">
+      <c r="G40">
         <v>94.200999999999993</v>
       </c>
     </row>
@@ -5118,13 +5131,13 @@
       <c r="D41">
         <v>96.343000000000004</v>
       </c>
-      <c r="E41" s="1">
+      <c r="E41">
         <v>97.837000000000003</v>
       </c>
-      <c r="F41" s="1">
+      <c r="F41">
         <v>96.129000000000005</v>
       </c>
-      <c r="G41" s="1">
+      <c r="G41">
         <v>94.212999999999994</v>
       </c>
     </row>
@@ -5141,13 +5154,13 @@
       <c r="D42">
         <v>96.353999999999999</v>
       </c>
-      <c r="E42" s="1">
+      <c r="E42">
         <v>97.846999999999994</v>
       </c>
-      <c r="F42" s="1">
+      <c r="F42">
         <v>96.137</v>
       </c>
-      <c r="G42" s="1">
+      <c r="G42">
         <v>94.221000000000004</v>
       </c>
     </row>
@@ -5164,13 +5177,13 @@
       <c r="D43">
         <v>96.355999999999995</v>
       </c>
-      <c r="E43" s="1">
+      <c r="E43">
         <v>98.009</v>
       </c>
-      <c r="F43" s="1">
+      <c r="F43">
         <v>97.168000000000006</v>
       </c>
-      <c r="G43" s="1">
+      <c r="G43">
         <v>88.335999999999999</v>
       </c>
     </row>
@@ -5187,13 +5200,13 @@
       <c r="D44">
         <v>96.367000000000004</v>
       </c>
-      <c r="E44" s="1">
+      <c r="E44">
         <v>98.147999999999996</v>
       </c>
-      <c r="F44" s="1">
+      <c r="F44">
         <v>97.402000000000001</v>
       </c>
-      <c r="G44" s="1">
+      <c r="G44">
         <v>89.751999999999995</v>
       </c>
     </row>
@@ -5210,13 +5223,13 @@
       <c r="D45">
         <v>96.655000000000001</v>
       </c>
-      <c r="E45" s="1">
+      <c r="E45">
         <v>96.117999999999995</v>
       </c>
-      <c r="F45" s="1">
+      <c r="F45">
         <v>93.959000000000003</v>
       </c>
-      <c r="G45" s="1">
+      <c r="G45">
         <v>90.870999999999995</v>
       </c>
     </row>
@@ -5233,13 +5246,13 @@
       <c r="D46">
         <v>96.878</v>
       </c>
-      <c r="E46" s="1">
+      <c r="E46">
         <v>96.450999999999993</v>
       </c>
-      <c r="F46" s="1">
+      <c r="F46">
         <v>94.528000000000006</v>
       </c>
-      <c r="G46" s="1">
+      <c r="G46">
         <v>91.771000000000001</v>
       </c>
     </row>
@@ -5256,13 +5269,13 @@
       <c r="D47">
         <v>97.054000000000002</v>
       </c>
-      <c r="E47" s="1">
+      <c r="E47">
         <v>96.710999999999999</v>
       </c>
-      <c r="F47" s="1">
+      <c r="F47">
         <v>94.984999999999999</v>
       </c>
-      <c r="G47" s="1">
+      <c r="G47">
         <v>92.503</v>
       </c>
     </row>
@@ -5279,13 +5292,13 @@
       <c r="D48">
         <v>97.194000000000003</v>
       </c>
-      <c r="E48" s="1">
+      <c r="E48">
         <v>96.915999999999997</v>
       </c>
-      <c r="F48" s="1">
+      <c r="F48">
         <v>95.353999999999999</v>
       </c>
-      <c r="G48" s="1">
+      <c r="G48">
         <v>93.106999999999999</v>
       </c>
     </row>
@@ -5302,13 +5315,13 @@
       <c r="D49">
         <v>97.305999999999997</v>
       </c>
-      <c r="E49" s="1">
+      <c r="E49">
         <v>97.078999999999994</v>
       </c>
-      <c r="F49" s="1">
+      <c r="F49">
         <v>95.656999999999996</v>
       </c>
-      <c r="G49" s="1">
+      <c r="G49">
         <v>93.611000000000004</v>
       </c>
     </row>
@@ -5325,13 +5338,13 @@
       <c r="D50">
         <v>97.397000000000006</v>
       </c>
-      <c r="E50" s="1">
+      <c r="E50">
         <v>97.209000000000003</v>
       </c>
-      <c r="F50" s="1">
+      <c r="F50">
         <v>95.906000000000006</v>
       </c>
-      <c r="G50" s="1">
+      <c r="G50">
         <v>94.033000000000001</v>
       </c>
     </row>
@@ -5348,13 +5361,13 @@
       <c r="D51">
         <v>97.47</v>
       </c>
-      <c r="E51" s="1">
+      <c r="E51">
         <v>97.313000000000002</v>
       </c>
-      <c r="F51" s="1">
+      <c r="F51">
         <v>96.111999999999995</v>
       </c>
-      <c r="G51" s="1">
+      <c r="G51">
         <v>94.391000000000005</v>
       </c>
     </row>
@@ -5371,13 +5384,13 @@
       <c r="D52">
         <v>97.528999999999996</v>
       </c>
-      <c r="E52" s="1">
+      <c r="E52">
         <v>97.394000000000005</v>
       </c>
-      <c r="F52" s="1">
+      <c r="F52">
         <v>96.284000000000006</v>
       </c>
-      <c r="G52" s="1">
+      <c r="G52">
         <v>94.694999999999993</v>
       </c>
     </row>
@@ -5394,13 +5407,13 @@
       <c r="D53">
         <v>97.575999999999993</v>
       </c>
-      <c r="E53" s="1">
+      <c r="E53">
         <v>97.456999999999994</v>
       </c>
-      <c r="F53" s="1">
+      <c r="F53">
         <v>96.426000000000002</v>
       </c>
-      <c r="G53" s="1">
+      <c r="G53">
         <v>94.953999999999994</v>
       </c>
     </row>
@@ -5417,13 +5430,13 @@
       <c r="D54">
         <v>97.613</v>
       </c>
-      <c r="E54" s="1">
+      <c r="E54">
         <v>97.506</v>
       </c>
-      <c r="F54" s="1">
+      <c r="F54">
         <v>96.543000000000006</v>
       </c>
-      <c r="G54" s="1">
+      <c r="G54">
         <v>95.176000000000002</v>
       </c>
     </row>
@@ -5440,13 +5453,13 @@
       <c r="D55">
         <v>97.641999999999996</v>
       </c>
-      <c r="E55" s="1">
+      <c r="E55">
         <v>97.540999999999997</v>
       </c>
-      <c r="F55" s="1">
+      <c r="F55">
         <v>96.64</v>
       </c>
-      <c r="G55" s="1">
+      <c r="G55">
         <v>95.367000000000004</v>
       </c>
     </row>
@@ -5463,13 +5476,13 @@
       <c r="D56">
         <v>97.662999999999997</v>
       </c>
-      <c r="E56" s="1">
+      <c r="E56">
         <v>97.566000000000003</v>
       </c>
-      <c r="F56" s="1">
+      <c r="F56">
         <v>96.72</v>
       </c>
-      <c r="G56" s="1">
+      <c r="G56">
         <v>95.53</v>
       </c>
     </row>
@@ -5486,13 +5499,13 @@
       <c r="D57">
         <v>97.688999999999993</v>
       </c>
-      <c r="E57" s="1">
+      <c r="E57">
         <v>97.587999999999994</v>
       </c>
-      <c r="F57" s="1">
+      <c r="F57">
         <v>96.835999999999999</v>
       </c>
-      <c r="G57" s="1">
+      <c r="G57">
         <v>95.789000000000001</v>
       </c>
     </row>
@@ -5509,13 +5522,13 @@
       <c r="D58">
         <v>97.694999999999993</v>
       </c>
-      <c r="E58" s="1">
+      <c r="E58">
         <v>97.582999999999998</v>
       </c>
-      <c r="F58" s="1">
+      <c r="F58">
         <v>96.906000000000006</v>
       </c>
-      <c r="G58" s="1">
+      <c r="G58">
         <v>95.977999999999994</v>
       </c>
     </row>
@@ -5532,13 +5545,13 @@
       <c r="D59">
         <v>97.688000000000002</v>
       </c>
-      <c r="E59" s="1">
+      <c r="E59">
         <v>97.555000000000007</v>
       </c>
-      <c r="F59" s="1">
+      <c r="F59">
         <v>96.941000000000003</v>
       </c>
-      <c r="G59" s="1">
+      <c r="G59">
         <v>96.111999999999995</v>
       </c>
     </row>
@@ -5555,13 +5568,13 @@
       <c r="D60">
         <v>97.668000000000006</v>
       </c>
-      <c r="E60" s="1">
+      <c r="E60">
         <v>97.509</v>
       </c>
-      <c r="F60" s="1">
+      <c r="F60">
         <v>96.947000000000003</v>
       </c>
-      <c r="G60" s="1">
+      <c r="G60">
         <v>96.201999999999998</v>
       </c>
     </row>
@@ -5578,13 +5591,13 @@
       <c r="D61">
         <v>97.64</v>
       </c>
-      <c r="E61" s="1">
+      <c r="E61">
         <v>97.448999999999998</v>
       </c>
-      <c r="F61" s="1">
+      <c r="F61">
         <v>96.93</v>
       </c>
-      <c r="G61" s="1">
+      <c r="G61">
         <v>96.257999999999996</v>
       </c>
     </row>
@@ -5601,13 +5614,13 @@
       <c r="D62">
         <v>97.603999999999999</v>
       </c>
-      <c r="E62" s="1">
+      <c r="E62">
         <v>97.376999999999995</v>
       </c>
-      <c r="F62" s="1">
+      <c r="F62">
         <v>96.894999999999996</v>
       </c>
-      <c r="G62" s="1">
+      <c r="G62">
         <v>96.284000000000006</v>
       </c>
     </row>
@@ -5624,13 +5637,13 @@
       <c r="D63">
         <v>97.561000000000007</v>
       </c>
-      <c r="E63" s="1">
+      <c r="E63">
         <v>97.293999999999997</v>
       </c>
-      <c r="F63" s="1">
+      <c r="F63">
         <v>96.843000000000004</v>
       </c>
-      <c r="G63" s="1">
+      <c r="G63">
         <v>96.286000000000001</v>
       </c>
     </row>
@@ -5647,13 +5660,13 @@
       <c r="D64">
         <v>97.513000000000005</v>
       </c>
-      <c r="E64" s="1">
+      <c r="E64">
         <v>97.201999999999998</v>
       </c>
-      <c r="F64" s="1">
+      <c r="F64">
         <v>96.778000000000006</v>
       </c>
-      <c r="G64" s="1">
+      <c r="G64">
         <v>96.268000000000001</v>
       </c>
     </row>
@@ -5670,13 +5683,13 @@
       <c r="D65">
         <v>97.46</v>
       </c>
-      <c r="E65" s="1">
+      <c r="E65">
         <v>97.100999999999999</v>
       </c>
-      <c r="F65" s="1">
+      <c r="F65">
         <v>96.7</v>
       </c>
-      <c r="G65" s="1">
+      <c r="G65">
         <v>96.231999999999999</v>
       </c>
     </row>
@@ -5693,13 +5706,13 @@
       <c r="D66">
         <v>97.403000000000006</v>
       </c>
-      <c r="E66" s="1">
+      <c r="E66">
         <v>96.992999999999995</v>
       </c>
-      <c r="F66" s="1">
+      <c r="F66">
         <v>96.611000000000004</v>
       </c>
-      <c r="G66" s="1">
+      <c r="G66">
         <v>96.180999999999997</v>
       </c>
     </row>

</xml_diff>